<commit_message>
#86 PCBWay BOM Review Completed.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark-BOM-v2.0 Boards)_PCWay.xlsx
+++ b/Deliverables/BOM/eSpark-BOM-v2.0 Boards)_PCWay.xlsx
@@ -1,35 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\Melih-SoundSensor\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Melih-SoundSensor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{211C0C1F-8B88-4ACF-9851-6FD70D8EC895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="240">
   <si>
     <t>S. No.</t>
   </si>
@@ -359,9 +350,6 @@
     <t>C98220</t>
   </si>
   <si>
-    <t>C2869734</t>
-  </si>
-  <si>
     <t>C86534</t>
   </si>
   <si>
@@ -597,9 +585,6 @@
     <t>33nF</t>
   </si>
   <si>
-    <t>C48260</t>
-  </si>
-  <si>
     <t>FIXED IND 3.3NH 1A 120 MOHM SMD</t>
   </si>
   <si>
@@ -621,9 +606,6 @@
     <t>LQG15HS1N2S02D</t>
   </si>
   <si>
-    <t>C162552</t>
-  </si>
-  <si>
     <t>C77105</t>
   </si>
   <si>
@@ -760,12 +742,15 @@
   </si>
   <si>
     <t>C2764612</t>
+  </si>
+  <si>
+    <t>C2972450</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
   </numFmts>
@@ -933,7 +918,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1190,6 +1175,103 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1199,7 +1281,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1226,9 +1308,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1277,9 +1356,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1289,16 +1365,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1310,9 +1377,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1322,9 +1386,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1343,12 +1404,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1358,15 +1413,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1382,15 +1431,6 @@
     <xf numFmtId="164" fontId="14" fillId="6" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1400,12 +1440,6 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1413,12 +1447,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1439,49 +1467,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1491,9 +1480,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1508,16 +1494,124 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1795,14 +1889,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="47.5703125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="32.28515625" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.5703125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="35.140625" style="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
@@ -1813,18 +1907,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16.5" thickBot="1">
-      <c r="A1" s="86" t="s">
-        <v>118</v>
-      </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87"/>
-      <c r="H1" s="87"/>
-      <c r="I1" s="87"/>
-      <c r="J1" s="87"/>
+      <c r="A1" s="74" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="88"/>
     </row>
     <row r="2" spans="1:11" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -1851,8 +1945,8 @@
       <c r="H2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="71" t="s">
-        <v>203</v>
+      <c r="I2" s="55" t="s">
+        <v>200</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>8</v>
@@ -1862,31 +1956,31 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="88" t="s">
+      <c r="B3" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="67" t="s">
-        <v>125</v>
-      </c>
-      <c r="E3" s="37" t="s">
+      <c r="D3" s="53" t="s">
+        <v>124</v>
+      </c>
+      <c r="E3" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="37" t="s">
+      <c r="F3" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="H3" s="36" t="s">
+      <c r="H3" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="16">
+      <c r="I3" s="15">
         <v>100</v>
       </c>
-      <c r="J3" s="38">
+      <c r="J3" s="89">
         <v>4</v>
       </c>
     </row>
@@ -1894,29 +1988,29 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="89"/>
-      <c r="C4" s="39" t="s">
+      <c r="B4" s="77"/>
+      <c r="C4" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="51" t="s">
+      <c r="D4" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="H4" s="40" t="s">
+      <c r="H4" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="I4" s="20">
+      <c r="I4" s="19">
         <v>40</v>
       </c>
-      <c r="J4" s="42">
+      <c r="J4" s="90">
         <v>1</v>
       </c>
     </row>
@@ -1924,29 +2018,29 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="89"/>
-      <c r="C5" s="39" t="s">
+      <c r="B5" s="77"/>
+      <c r="C5" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="66" t="s">
-        <v>121</v>
-      </c>
-      <c r="E5" s="40" t="s">
+      <c r="D5" s="52" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="H5" s="40" t="s">
+      <c r="H5" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="20">
+      <c r="I5" s="19">
         <v>400</v>
       </c>
-      <c r="J5" s="42">
+      <c r="J5" s="90">
         <v>19</v>
       </c>
       <c r="K5" s="9"/>
@@ -1955,29 +2049,29 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="89"/>
-      <c r="C6" s="39" t="s">
+      <c r="B6" s="77"/>
+      <c r="C6" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="51" t="s">
+      <c r="D6" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="41" t="s">
+      <c r="E6" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="20">
+      <c r="I6" s="19">
         <v>200</v>
       </c>
-      <c r="J6" s="42">
+      <c r="J6" s="90">
         <v>8</v>
       </c>
       <c r="K6" s="9"/>
@@ -1986,29 +2080,29 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="89"/>
-      <c r="C7" s="39" t="s">
+      <c r="B7" s="77"/>
+      <c r="C7" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="D7" s="51" t="s">
+      <c r="E7" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="41" t="s">
-        <v>124</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="G7" s="18" t="s">
+      <c r="F7" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="H7" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="H7" s="40" t="s">
-        <v>157</v>
-      </c>
-      <c r="I7" s="20">
+      <c r="I7" s="19">
         <v>100</v>
       </c>
-      <c r="J7" s="42">
+      <c r="J7" s="90">
         <v>1</v>
       </c>
       <c r="K7" s="9"/>
@@ -2017,29 +2111,29 @@
       <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="89"/>
-      <c r="C8" s="39" t="s">
+      <c r="B8" s="77"/>
+      <c r="C8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="66" t="s">
-        <v>173</v>
-      </c>
-      <c r="E8" s="40" t="s">
+      <c r="D8" s="52" t="s">
+        <v>172</v>
+      </c>
+      <c r="E8" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="H8" s="40" t="s">
+      <c r="H8" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="20">
+      <c r="I8" s="19">
         <v>600</v>
       </c>
-      <c r="J8" s="42">
+      <c r="J8" s="90">
         <v>29</v>
       </c>
       <c r="K8" s="9"/>
@@ -2048,29 +2142,29 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="89"/>
-      <c r="C9" s="39" t="s">
+      <c r="B9" s="77"/>
+      <c r="C9" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="51" t="s">
+      <c r="D9" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="F9" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="G9" s="22" t="s">
+      <c r="G9" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="H9" s="40" t="s">
+      <c r="H9" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="I9" s="21">
+      <c r="I9" s="20">
         <v>30</v>
       </c>
-      <c r="J9" s="42">
+      <c r="J9" s="90">
         <v>1</v>
       </c>
       <c r="K9" s="9"/>
@@ -2079,60 +2173,60 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="89"/>
-      <c r="C10" s="39" t="s">
+      <c r="B10" s="77"/>
+      <c r="C10" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="51" t="s">
+      <c r="D10" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="41" t="s">
+      <c r="F10" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="40" t="s">
+      <c r="H10" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="I10" s="21">
+      <c r="I10" s="20">
         <v>200</v>
       </c>
-      <c r="J10" s="42">
+      <c r="J10" s="90">
         <v>6</v>
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="39" thickBot="1">
+    <row r="11" spans="1:11" ht="26.25" thickBot="1">
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="89"/>
-      <c r="C11" s="39" t="s">
+      <c r="B11" s="77"/>
+      <c r="C11" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="66" t="s">
+      <c r="D11" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="40" t="s">
+      <c r="E11" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="40" t="s">
+      <c r="F11" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="G11" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="H11" s="40" t="s">
+      <c r="H11" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="I11" s="21">
+      <c r="I11" s="20">
         <v>350</v>
       </c>
-      <c r="J11" s="42">
+      <c r="J11" s="90">
         <v>16</v>
       </c>
       <c r="K11" s="9"/>
@@ -2141,29 +2235,29 @@
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="89"/>
-      <c r="C12" s="39" t="s">
+      <c r="B12" s="77"/>
+      <c r="C12" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="D12" s="51" t="s">
+      <c r="E12" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="E12" s="41" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="41" t="s">
-        <v>128</v>
-      </c>
-      <c r="G12" s="18" t="s">
+      <c r="G12" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="H12" s="34" t="s">
         <v>158</v>
       </c>
-      <c r="H12" s="40" t="s">
-        <v>159</v>
-      </c>
-      <c r="I12" s="21">
+      <c r="I12" s="20">
         <v>50</v>
       </c>
-      <c r="J12" s="42">
+      <c r="J12" s="90">
         <v>1</v>
       </c>
       <c r="K12" s="9"/>
@@ -2172,29 +2266,29 @@
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="89"/>
-      <c r="C13" s="39" t="s">
+      <c r="B13" s="77"/>
+      <c r="C13" s="33" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="D13" s="66" t="s">
-        <v>130</v>
-      </c>
-      <c r="E13" s="40" t="s">
-        <v>124</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="G13" s="18" t="s">
+      <c r="E13" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="H13" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="H13" s="40" t="s">
-        <v>161</v>
-      </c>
-      <c r="I13" s="21">
+      <c r="I13" s="20">
         <v>100</v>
       </c>
-      <c r="J13" s="42">
+      <c r="J13" s="90">
         <v>1</v>
       </c>
       <c r="K13" s="9"/>
@@ -2203,29 +2297,29 @@
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="89"/>
-      <c r="C14" s="39" t="s">
+      <c r="B14" s="77"/>
+      <c r="C14" s="33" t="s">
+        <v>173</v>
+      </c>
+      <c r="D14" s="42" t="s">
         <v>174</v>
       </c>
-      <c r="D14" s="51" t="s">
+      <c r="E14" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="E14" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="F14" s="41" t="s">
-        <v>176</v>
-      </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="H14" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="H14" s="40" t="s">
-        <v>184</v>
-      </c>
-      <c r="I14" s="21">
+      <c r="I14" s="20">
         <v>100</v>
       </c>
-      <c r="J14" s="42">
+      <c r="J14" s="90">
         <v>1</v>
       </c>
       <c r="K14" s="9"/>
@@ -2234,29 +2328,29 @@
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="89"/>
-      <c r="C15" s="39" t="s">
+      <c r="B15" s="77"/>
+      <c r="C15" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="D15" s="42" t="s">
         <v>177</v>
       </c>
-      <c r="D15" s="51" t="s">
+      <c r="E15" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="35" t="s">
         <v>178</v>
       </c>
-      <c r="E15" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="F15" s="41" t="s">
-        <v>179</v>
-      </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="H15" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="H15" s="40" t="s">
-        <v>186</v>
-      </c>
-      <c r="I15" s="21">
+      <c r="I15" s="20">
         <v>50</v>
       </c>
-      <c r="J15" s="42">
+      <c r="J15" s="90">
         <v>2</v>
       </c>
       <c r="K15" s="9"/>
@@ -2265,29 +2359,29 @@
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="89"/>
-      <c r="C16" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>207</v>
-      </c>
-      <c r="E16" s="41" t="s">
+      <c r="B16" s="77"/>
+      <c r="C16" s="33" t="s">
+        <v>203</v>
+      </c>
+      <c r="D16" s="42" t="s">
+        <v>204</v>
+      </c>
+      <c r="E16" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="41" t="s">
-        <v>208</v>
-      </c>
-      <c r="G16" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="H16" s="40" t="s">
-        <v>213</v>
-      </c>
-      <c r="I16" s="21">
+      <c r="F16" s="35" t="s">
+        <v>205</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="H16" s="34" t="s">
+        <v>210</v>
+      </c>
+      <c r="I16" s="20">
         <v>50</v>
       </c>
-      <c r="J16" s="42">
+      <c r="J16" s="90">
         <v>1</v>
       </c>
       <c r="K16" s="9"/>
@@ -2296,29 +2390,29 @@
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="90"/>
-      <c r="C17" s="55" t="s">
-        <v>209</v>
-      </c>
-      <c r="D17" s="30" t="s">
-        <v>210</v>
-      </c>
-      <c r="E17" s="65" t="s">
+      <c r="B17" s="78"/>
+      <c r="C17" s="45" t="s">
+        <v>206</v>
+      </c>
+      <c r="D17" s="54" t="s">
+        <v>207</v>
+      </c>
+      <c r="E17" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="F17" s="65" t="s">
+      <c r="F17" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="G17" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="G17" s="29" t="s">
-        <v>214</v>
-      </c>
-      <c r="H17" s="47" t="s">
-        <v>215</v>
-      </c>
-      <c r="I17" s="28">
+      <c r="H17" s="40" t="s">
+        <v>212</v>
+      </c>
+      <c r="I17" s="26">
         <v>50</v>
       </c>
-      <c r="J17" s="49">
+      <c r="J17" s="91">
         <v>1</v>
       </c>
       <c r="K17" s="9"/>
@@ -2327,31 +2421,31 @@
       <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="91" t="s">
-        <v>150</v>
-      </c>
-      <c r="C18" s="75" t="s">
+      <c r="B18" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="C18" s="57" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" s="53" t="s">
         <v>147</v>
       </c>
-      <c r="D18" s="67" t="s">
+      <c r="E18" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="F18" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="E18" s="36" t="s">
+      <c r="G18" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="36" t="s">
-        <v>149</v>
-      </c>
-      <c r="G18" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="H18" s="36" t="s">
+      <c r="H18" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="I18" s="14">
+      <c r="I18" s="13">
         <v>30</v>
       </c>
-      <c r="J18" s="38">
+      <c r="J18" s="89">
         <v>1</v>
       </c>
       <c r="K18" s="9"/>
@@ -2360,29 +2454,29 @@
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="92"/>
-      <c r="C19" s="76" t="s">
+      <c r="B19" s="80"/>
+      <c r="C19" s="58" t="s">
+        <v>179</v>
+      </c>
+      <c r="D19" s="54" t="s">
         <v>180</v>
       </c>
-      <c r="D19" s="70" t="s">
+      <c r="E19" s="40" t="s">
+        <v>22</v>
+      </c>
+      <c r="F19" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="E19" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="G19" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="H19" s="47" t="s">
+      <c r="G19" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="H19" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="I19" s="28">
-        <v>45</v>
-      </c>
-      <c r="J19" s="49">
+      <c r="I19" s="26">
+        <v>50</v>
+      </c>
+      <c r="J19" s="91">
         <v>2</v>
       </c>
       <c r="K19" s="9"/>
@@ -2391,31 +2485,31 @@
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="95" t="s">
-        <v>155</v>
-      </c>
-      <c r="C20" s="35" t="s">
+      <c r="B20" s="83" t="s">
+        <v>154</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="D20" s="53" t="s">
         <v>151</v>
       </c>
-      <c r="D20" s="67" t="s">
+      <c r="E20" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="E20" s="37" t="s">
+      <c r="F20" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="F20" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="H20" s="36" t="s">
+      <c r="G20" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="H20" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="I20" s="14">
+      <c r="I20" s="13">
         <v>50</v>
       </c>
-      <c r="J20" s="38">
+      <c r="J20" s="89">
         <v>1</v>
       </c>
       <c r="K20" s="9"/>
@@ -2424,29 +2518,29 @@
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="93"/>
-      <c r="C21" s="39" t="s">
+      <c r="B21" s="81"/>
+      <c r="C21" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="E21" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="F21" s="35" t="s">
         <v>188</v>
       </c>
-      <c r="D21" s="51" t="s">
-        <v>189</v>
-      </c>
-      <c r="E21" s="41" t="s">
-        <v>153</v>
-      </c>
-      <c r="F21" s="41" t="s">
-        <v>190</v>
-      </c>
       <c r="G21" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="H21" s="40" t="s">
-        <v>168</v>
-      </c>
-      <c r="I21" s="21">
-        <v>50</v>
-      </c>
-      <c r="J21" s="42">
+        <v>31</v>
+      </c>
+      <c r="H21" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="I21" s="20">
+        <v>45</v>
+      </c>
+      <c r="J21" s="90">
         <v>2</v>
       </c>
       <c r="K21" s="9"/>
@@ -2455,29 +2549,29 @@
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="93"/>
-      <c r="C22" s="39" t="s">
+      <c r="B22" s="81"/>
+      <c r="C22" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="D22" s="42" t="s">
+        <v>190</v>
+      </c>
+      <c r="E22" s="35" t="s">
         <v>191</v>
       </c>
-      <c r="D22" s="51" t="s">
+      <c r="F22" s="35" t="s">
         <v>192</v>
       </c>
-      <c r="E22" s="41" t="s">
+      <c r="G22" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="F22" s="41" t="s">
-        <v>194</v>
-      </c>
-      <c r="G22" s="18" t="s">
-        <v>196</v>
-      </c>
-      <c r="H22" s="40" t="s">
-        <v>168</v>
-      </c>
-      <c r="I22" s="21">
+      <c r="H22" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="I22" s="20">
         <v>50</v>
       </c>
-      <c r="J22" s="42">
+      <c r="J22" s="90">
         <v>2</v>
       </c>
       <c r="K22" s="9"/>
@@ -2486,29 +2580,29 @@
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="94"/>
-      <c r="C23" s="55" t="s">
+      <c r="B23" s="82"/>
+      <c r="C23" s="45" t="s">
+        <v>213</v>
+      </c>
+      <c r="D23" s="54" t="s">
+        <v>214</v>
+      </c>
+      <c r="E23" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="51" t="s">
+        <v>215</v>
+      </c>
+      <c r="G23" s="27" t="s">
         <v>216</v>
       </c>
-      <c r="D23" s="30" t="s">
-        <v>217</v>
-      </c>
-      <c r="E23" s="65" t="s">
-        <v>22</v>
-      </c>
-      <c r="F23" s="65" t="s">
-        <v>218</v>
-      </c>
-      <c r="G23" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="H23" s="47" t="s">
-        <v>168</v>
-      </c>
-      <c r="I23" s="28">
+      <c r="H23" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="I23" s="26">
         <v>30</v>
       </c>
-      <c r="J23" s="49">
+      <c r="J23" s="91">
         <v>1</v>
       </c>
       <c r="K23" s="9"/>
@@ -2517,31 +2611,31 @@
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="68" t="s">
+      <c r="B24" s="64" t="s">
         <v>62</v>
       </c>
-      <c r="C24" s="97" t="s">
+      <c r="C24" s="66" t="s">
         <v>59</v>
       </c>
-      <c r="D24" s="98" t="s">
+      <c r="D24" s="85" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="99" t="s">
+      <c r="E24" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="99" t="s">
+      <c r="F24" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="100" t="s">
-        <v>116</v>
-      </c>
-      <c r="H24" s="99" t="s">
+      <c r="G24" s="68" t="s">
+        <v>115</v>
+      </c>
+      <c r="H24" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="I24" s="99">
+      <c r="I24" s="67">
         <v>162</v>
       </c>
-      <c r="J24" s="74">
+      <c r="J24" s="92">
         <v>8</v>
       </c>
       <c r="K24" s="9"/>
@@ -2550,31 +2644,31 @@
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="69" t="s">
+      <c r="B25" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="53" t="s">
+      <c r="C25" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="D25" s="73" t="s">
+      <c r="D25" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="43" t="s">
+      <c r="E25" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="F25" s="43" t="s">
+      <c r="F25" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="G25" s="24" t="s">
+      <c r="G25" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="72" t="s">
+      <c r="H25" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="I25" s="72">
+      <c r="I25" s="56">
         <v>30</v>
       </c>
-      <c r="J25" s="56">
+      <c r="J25" s="93">
         <v>1</v>
       </c>
       <c r="K25" s="9"/>
@@ -2583,31 +2677,31 @@
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="88" t="s">
+      <c r="B26" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="44" t="s">
+      <c r="C26" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="D26" s="45" t="s">
+      <c r="D26" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="E26" s="45" t="s">
+      <c r="E26" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="45" t="s">
+      <c r="F26" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="G26" s="25" t="s">
+      <c r="G26" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="H26" s="26" t="s">
+      <c r="H26" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="I26" s="26">
-        <v>23</v>
-      </c>
-      <c r="J26" s="27">
+      <c r="I26" s="25">
+        <v>22</v>
+      </c>
+      <c r="J26" s="94">
         <v>1</v>
       </c>
       <c r="K26" s="9"/>
@@ -2616,29 +2710,29 @@
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="89"/>
-      <c r="C27" s="48" t="s">
+      <c r="B27" s="77"/>
+      <c r="C27" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="D27" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="40" t="s">
+      <c r="E27" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="F27" s="40" t="s">
+      <c r="F27" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="G27" s="18" t="s">
+      <c r="G27" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="H27" s="20" t="s">
+      <c r="H27" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I27" s="20">
+      <c r="I27" s="19">
         <v>45</v>
       </c>
-      <c r="J27" s="54">
+      <c r="J27" s="95">
         <v>2</v>
       </c>
       <c r="K27" s="9"/>
@@ -2647,29 +2741,29 @@
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="90"/>
-      <c r="C28" s="46" t="s">
+      <c r="B28" s="78"/>
+      <c r="C28" s="39" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="D28" s="64" t="s">
+      <c r="E28" s="40" t="s">
+        <v>22</v>
+      </c>
+      <c r="F28" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="E28" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="F28" s="47" t="s">
-        <v>133</v>
-      </c>
-      <c r="G28" s="29" t="s">
+      <c r="G28" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="H28" s="28" t="s">
         <v>167</v>
       </c>
-      <c r="H28" s="30" t="s">
-        <v>168</v>
-      </c>
-      <c r="I28" s="30">
+      <c r="I28" s="28">
         <v>25</v>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="96">
         <v>1</v>
       </c>
       <c r="K28" s="9"/>
@@ -2678,31 +2772,31 @@
       <c r="A29" s="6">
         <v>27</v>
       </c>
-      <c r="B29" s="88" t="s">
+      <c r="B29" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="44" t="s">
+      <c r="C29" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="D29" s="77" t="s">
-        <v>134</v>
-      </c>
-      <c r="E29" s="36" t="s">
+      <c r="D29" s="59" t="s">
+        <v>133</v>
+      </c>
+      <c r="E29" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="F29" s="67" t="s">
+      <c r="F29" s="53" t="s">
         <v>106</v>
       </c>
-      <c r="G29" s="15" t="s">
+      <c r="G29" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="H29" s="36" t="s">
+      <c r="H29" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="I29" s="78">
+      <c r="I29" s="60">
         <v>100</v>
       </c>
-      <c r="J29" s="78">
+      <c r="J29" s="97">
         <v>3</v>
       </c>
       <c r="K29" s="9"/>
@@ -2711,29 +2805,29 @@
       <c r="A30" s="6">
         <v>28</v>
       </c>
-      <c r="B30" s="89"/>
-      <c r="C30" s="48" t="s">
-        <v>221</v>
-      </c>
-      <c r="D30" s="85" t="s">
-        <v>135</v>
-      </c>
-      <c r="E30" s="40" t="s">
+      <c r="B30" s="77"/>
+      <c r="C30" s="41" t="s">
+        <v>218</v>
+      </c>
+      <c r="D30" s="52" t="s">
+        <v>134</v>
+      </c>
+      <c r="E30" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="F30" s="40" t="s">
-        <v>222</v>
-      </c>
-      <c r="G30" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="H30" s="40" t="s">
+      <c r="F30" s="34" t="s">
+        <v>219</v>
+      </c>
+      <c r="G30" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="I30" s="52">
+      <c r="H30" s="34" t="s">
+        <v>217</v>
+      </c>
+      <c r="I30" s="43">
         <v>100</v>
       </c>
-      <c r="J30" s="52">
+      <c r="J30" s="98">
         <v>1</v>
       </c>
       <c r="K30" s="9"/>
@@ -2742,29 +2836,29 @@
       <c r="A31" s="6">
         <v>29</v>
       </c>
-      <c r="B31" s="89"/>
-      <c r="C31" s="48" t="s">
+      <c r="B31" s="77"/>
+      <c r="C31" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="D31" s="52" t="s">
         <v>136</v>
       </c>
-      <c r="D31" s="66" t="s">
+      <c r="E31" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="34" t="s">
         <v>137</v>
       </c>
-      <c r="E31" s="40" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="40" t="s">
+      <c r="G31" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="H31" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="G31" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="H31" s="40" t="s">
-        <v>139</v>
-      </c>
-      <c r="I31" s="52">
+      <c r="I31" s="43">
         <v>100</v>
       </c>
-      <c r="J31" s="52">
+      <c r="J31" s="98">
         <v>1</v>
       </c>
       <c r="K31" s="9"/>
@@ -2773,29 +2867,29 @@
       <c r="A32" s="6">
         <v>30</v>
       </c>
-      <c r="B32" s="89"/>
-      <c r="C32" s="48" t="s">
+      <c r="B32" s="77"/>
+      <c r="C32" s="41" t="s">
+        <v>194</v>
+      </c>
+      <c r="D32" s="52" t="s">
+        <v>195</v>
+      </c>
+      <c r="E32" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="G32" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="D32" s="66" t="s">
+      <c r="H32" s="34" t="s">
         <v>198</v>
       </c>
-      <c r="E32" s="40" t="s">
-        <v>18</v>
-      </c>
-      <c r="F32" s="40" t="s">
-        <v>199</v>
-      </c>
-      <c r="G32" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="H32" s="40" t="s">
-        <v>201</v>
-      </c>
-      <c r="I32" s="52">
+      <c r="I32" s="43">
         <v>100</v>
       </c>
-      <c r="J32" s="52">
+      <c r="J32" s="98">
         <v>4</v>
       </c>
       <c r="K32" s="9"/>
@@ -2804,29 +2898,29 @@
       <c r="A33" s="6">
         <v>31</v>
       </c>
-      <c r="B33" s="90"/>
-      <c r="C33" s="46" t="s">
+      <c r="B33" s="78"/>
+      <c r="C33" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="D33" s="79" t="s">
-        <v>231</v>
-      </c>
-      <c r="E33" s="47" t="s">
+      <c r="D33" s="61" t="s">
+        <v>228</v>
+      </c>
+      <c r="E33" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="F33" s="47" t="s">
+      <c r="F33" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="G33" s="29" t="s">
+      <c r="G33" s="27" t="s">
         <v>108</v>
       </c>
-      <c r="H33" s="47" t="s">
+      <c r="H33" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="I33" s="80">
+      <c r="I33" s="62">
         <v>100</v>
       </c>
-      <c r="J33" s="80">
+      <c r="J33" s="99">
         <v>2</v>
       </c>
       <c r="K33" s="9"/>
@@ -2835,31 +2929,31 @@
       <c r="A34" s="6">
         <v>32</v>
       </c>
-      <c r="B34" s="88" t="s">
+      <c r="B34" s="76" t="s">
         <v>90</v>
       </c>
-      <c r="C34" s="44" t="s">
+      <c r="C34" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="D34" s="45" t="s">
+      <c r="D34" s="59" t="s">
         <v>75</v>
       </c>
-      <c r="E34" s="36" t="s">
+      <c r="E34" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="F34" s="36" t="s">
+      <c r="F34" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="G34" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="H34" s="16" t="s">
+      <c r="G34" s="84" t="s">
+        <v>30</v>
+      </c>
+      <c r="H34" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="I34" s="16">
+      <c r="I34" s="15">
         <v>42</v>
       </c>
-      <c r="J34" s="38">
+      <c r="J34" s="89">
         <v>2</v>
       </c>
       <c r="K34" s="9"/>
@@ -2868,29 +2962,29 @@
       <c r="A35" s="6">
         <v>33</v>
       </c>
-      <c r="B35" s="89"/>
-      <c r="C35" s="48" t="s">
+      <c r="B35" s="77"/>
+      <c r="C35" s="41" t="s">
         <v>78</v>
       </c>
-      <c r="D35" s="63" t="s">
+      <c r="D35" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="E35" s="40" t="s">
+      <c r="E35" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="F35" s="40" t="s">
+      <c r="F35" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="G35" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="H35" s="20" t="s">
+      <c r="G35" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="H35" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I35" s="19">
+      <c r="I35" s="18">
         <v>21</v>
       </c>
-      <c r="J35" s="42">
+      <c r="J35" s="90">
         <v>1</v>
       </c>
       <c r="K35" s="9"/>
@@ -2899,29 +2993,29 @@
       <c r="A36" s="6">
         <v>34</v>
       </c>
-      <c r="B36" s="89"/>
-      <c r="C36" s="48" t="s">
+      <c r="B36" s="77"/>
+      <c r="C36" s="41" t="s">
         <v>81</v>
       </c>
-      <c r="D36" s="63" t="s">
+      <c r="D36" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="E36" s="40" t="s">
+      <c r="E36" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="F36" s="40" t="s">
+      <c r="F36" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="G36" s="21" t="s">
+      <c r="G36" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="H36" s="20" t="s">
+      <c r="H36" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I36" s="21">
+      <c r="I36" s="20">
         <v>21</v>
       </c>
-      <c r="J36" s="42">
+      <c r="J36" s="90">
         <v>1</v>
       </c>
       <c r="K36" s="9"/>
@@ -2930,29 +3024,29 @@
       <c r="A37" s="6">
         <v>35</v>
       </c>
-      <c r="B37" s="89"/>
-      <c r="C37" s="101" t="s">
+      <c r="B37" s="77"/>
+      <c r="C37" s="69" t="s">
         <v>84</v>
       </c>
-      <c r="D37" s="85" t="s">
+      <c r="D37" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="E37" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="F37" s="20" t="s">
+      <c r="E37" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="F37" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="G37" s="21" t="s">
+      <c r="G37" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="H37" s="20" t="s">
+      <c r="H37" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I37" s="21">
+      <c r="I37" s="20">
         <v>41</v>
       </c>
-      <c r="J37" s="50">
+      <c r="J37" s="100">
         <v>2</v>
       </c>
       <c r="K37" s="9"/>
@@ -2961,29 +3055,29 @@
       <c r="A38" s="6">
         <v>36</v>
       </c>
-      <c r="B38" s="89"/>
-      <c r="C38" s="48" t="s">
+      <c r="B38" s="77"/>
+      <c r="C38" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="D38" s="52" t="s">
         <v>140</v>
       </c>
-      <c r="D38" s="63" t="s">
+      <c r="E38" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="F38" s="34" t="s">
         <v>141</v>
       </c>
-      <c r="E38" s="40" t="s">
+      <c r="G38" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="F38" s="40" t="s">
-        <v>142</v>
-      </c>
-      <c r="G38" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="H38" s="20" t="s">
+      <c r="H38" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I38" s="21">
+      <c r="I38" s="20">
         <v>21</v>
       </c>
-      <c r="J38" s="42">
+      <c r="J38" s="90">
         <v>1</v>
       </c>
       <c r="K38" s="9"/>
@@ -2992,29 +3086,29 @@
       <c r="A39" s="6">
         <v>37</v>
       </c>
-      <c r="B39" s="89"/>
-      <c r="C39" s="48" t="s">
+      <c r="B39" s="77"/>
+      <c r="C39" s="41" t="s">
+        <v>142</v>
+      </c>
+      <c r="D39" s="52" t="s">
         <v>143</v>
       </c>
-      <c r="D39" s="63" t="s">
+      <c r="E39" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="E39" s="40" t="s">
+      <c r="F39" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="F39" s="40" t="s">
-        <v>146</v>
-      </c>
-      <c r="G39" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="H39" s="20" t="s">
+      <c r="G39" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="H39" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I39" s="21">
+      <c r="I39" s="20">
         <v>21</v>
       </c>
-      <c r="J39" s="42">
+      <c r="J39" s="90">
         <v>1</v>
       </c>
       <c r="K39" s="9"/>
@@ -3023,333 +3117,341 @@
       <c r="A40" s="6">
         <v>38</v>
       </c>
-      <c r="B40" s="89"/>
-      <c r="C40" s="48" t="s">
-        <v>224</v>
-      </c>
-      <c r="D40" s="85" t="s">
-        <v>225</v>
-      </c>
-      <c r="E40" s="40" t="s">
+      <c r="B40" s="77"/>
+      <c r="C40" s="41" t="s">
+        <v>221</v>
+      </c>
+      <c r="D40" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="E40" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="F40" s="40" t="s">
-        <v>226</v>
-      </c>
-      <c r="G40" s="21"/>
-      <c r="H40" s="20" t="s">
+      <c r="F40" s="34" t="s">
+        <v>223</v>
+      </c>
+      <c r="G40" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="H40" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I40" s="21"/>
-      <c r="J40" s="42">
+      <c r="I40" s="20">
+        <v>22</v>
+      </c>
+      <c r="J40" s="90">
         <v>1</v>
       </c>
       <c r="K40" s="9"/>
     </row>
     <row r="41" spans="1:11" ht="15.75" thickBot="1">
-      <c r="A41" s="6"/>
-      <c r="B41" s="89"/>
-      <c r="C41" s="53" t="s">
-        <v>234</v>
-      </c>
-      <c r="D41" s="82" t="s">
+      <c r="A41" s="6">
+        <v>39</v>
+      </c>
+      <c r="B41" s="77"/>
+      <c r="C41" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="D41" s="86" t="s">
+        <v>229</v>
+      </c>
+      <c r="E41" s="36" t="s">
         <v>232</v>
       </c>
-      <c r="E41" s="43" t="s">
-        <v>235</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="G41" s="23" t="s">
+      <c r="F41" s="101" t="s">
+        <v>233</v>
+      </c>
+      <c r="G41" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="H41" s="20" t="s">
+      <c r="H41" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I41" s="23">
+      <c r="I41" s="22">
         <v>30</v>
       </c>
-      <c r="J41" s="81">
+      <c r="J41" s="102">
         <v>1</v>
       </c>
       <c r="K41" s="9"/>
     </row>
     <row r="42" spans="1:11" ht="26.25" thickBot="1">
       <c r="A42" s="6">
-        <v>39</v>
-      </c>
-      <c r="B42" s="90"/>
-      <c r="C42" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="78"/>
+      <c r="C42" s="39" t="s">
         <v>87</v>
       </c>
-      <c r="D42" s="64" t="s">
+      <c r="D42" s="61" t="s">
         <v>88</v>
       </c>
-      <c r="E42" s="47" t="s">
+      <c r="E42" s="40" t="s">
+        <v>111</v>
+      </c>
+      <c r="F42" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="G42" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="F42" s="47" t="s">
-        <v>89</v>
-      </c>
-      <c r="G42" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="H42" s="30" t="s">
+      <c r="H42" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="I42" s="28">
+      <c r="I42" s="26">
         <v>30</v>
       </c>
-      <c r="J42" s="49">
+      <c r="J42" s="91">
         <v>1</v>
       </c>
       <c r="K42" s="9"/>
     </row>
     <row r="43" spans="1:11" ht="15.75" thickBot="1">
       <c r="A43" s="6">
-        <v>40</v>
-      </c>
-      <c r="B43" s="88" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" s="76" t="s">
         <v>94</v>
       </c>
-      <c r="C43" s="44" t="s">
+      <c r="C43" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="D43" s="45" t="s">
+      <c r="D43" s="59" t="s">
         <v>32</v>
       </c>
-      <c r="E43" s="36" t="s">
+      <c r="E43" s="110" t="s">
         <v>22</v>
       </c>
-      <c r="F43" s="96" t="s">
+      <c r="F43" s="65" t="s">
         <v>92</v>
       </c>
-      <c r="G43" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="H43" s="16" t="s">
+      <c r="G43" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="H43" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="I43" s="32">
+      <c r="I43" s="29">
         <v>50</v>
       </c>
-      <c r="J43" s="33">
+      <c r="J43" s="103">
         <v>1</v>
       </c>
       <c r="K43" s="9"/>
     </row>
     <row r="44" spans="1:11" ht="26.25" thickBot="1">
       <c r="A44" s="6">
-        <v>41</v>
-      </c>
-      <c r="B44" s="89"/>
-      <c r="C44" s="48" t="s">
-        <v>239</v>
-      </c>
-      <c r="D44" s="63" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="77"/>
+      <c r="C44" s="41" t="s">
+        <v>236</v>
+      </c>
+      <c r="D44" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="E44" s="36" t="s">
+      <c r="E44" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="F44" s="40" t="s">
-        <v>240</v>
-      </c>
-      <c r="G44" s="20" t="s">
-        <v>241</v>
-      </c>
-      <c r="H44" s="20" t="s">
+      <c r="F44" s="34" t="s">
+        <v>237</v>
+      </c>
+      <c r="G44" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="H44" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I44" s="20">
+      <c r="I44" s="19">
         <v>30</v>
       </c>
-      <c r="J44" s="34">
+      <c r="J44" s="104">
         <v>1</v>
       </c>
       <c r="K44" s="9"/>
     </row>
     <row r="45" spans="1:11" ht="15.75" thickBot="1">
       <c r="A45" s="6">
-        <v>42</v>
-      </c>
-      <c r="B45" s="89"/>
-      <c r="C45" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="77"/>
+      <c r="C45" s="41" t="s">
         <v>93</v>
       </c>
-      <c r="D45" s="63" t="s">
+      <c r="D45" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="E45" s="40" t="s">
+      <c r="E45" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="F45" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="G45" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="H45" s="20" t="s">
+      <c r="F45" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="G45" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="H45" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I45" s="20">
+      <c r="I45" s="19">
         <v>50</v>
       </c>
-      <c r="J45" s="34">
+      <c r="J45" s="104">
         <v>1</v>
       </c>
       <c r="K45" s="9"/>
     </row>
     <row r="46" spans="1:11" ht="15.75" thickBot="1">
       <c r="A46" s="6">
-        <v>43</v>
-      </c>
-      <c r="B46" s="89"/>
-      <c r="C46" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="77"/>
+      <c r="C46" s="41" t="s">
+        <v>224</v>
+      </c>
+      <c r="D46" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="E46" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="F46" s="34" t="s">
+        <v>226</v>
+      </c>
+      <c r="G46" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="D46" s="85" t="s">
-        <v>228</v>
-      </c>
-      <c r="E46" s="40" t="s">
+      <c r="H46" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46" s="19">
+        <v>25</v>
+      </c>
+      <c r="J46" s="104">
+        <v>1</v>
+      </c>
+      <c r="K46" s="9"/>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" thickBot="1">
+      <c r="A47" s="6">
+        <v>45</v>
+      </c>
+      <c r="B47" s="77"/>
+      <c r="C47" s="44" t="s">
+        <v>234</v>
+      </c>
+      <c r="D47" s="87" t="s">
+        <v>230</v>
+      </c>
+      <c r="E47" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="F46" s="40" t="s">
-        <v>229</v>
-      </c>
-      <c r="G46" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="H46" s="20" t="s">
+      <c r="F47" s="105">
+        <v>61300611121</v>
+      </c>
+      <c r="G47" s="56" t="s">
+        <v>235</v>
+      </c>
+      <c r="H47" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="I46" s="20">
-        <v>25</v>
-      </c>
-      <c r="J46" s="34">
+      <c r="I47" s="56">
+        <v>40</v>
+      </c>
+      <c r="J47" s="106">
         <v>1</v>
       </c>
-      <c r="K46" s="9"/>
-    </row>
-    <row r="47" spans="1:11" ht="15.75" thickBot="1">
-      <c r="A47" s="6"/>
-      <c r="B47" s="89"/>
-      <c r="C47" s="53" t="s">
-        <v>237</v>
-      </c>
-      <c r="D47" s="43" t="s">
-        <v>233</v>
-      </c>
-      <c r="E47" s="40" t="s">
-        <v>22</v>
-      </c>
-      <c r="F47" s="84">
-        <v>61300611121</v>
-      </c>
-      <c r="G47" s="72" t="s">
-        <v>238</v>
-      </c>
-      <c r="H47" s="20" t="s">
+      <c r="K47" s="9"/>
+    </row>
+    <row r="48" spans="1:11" ht="102.75" thickBot="1">
+      <c r="A48" s="6">
+        <v>46</v>
+      </c>
+      <c r="B48" s="78"/>
+      <c r="C48" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="D48" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="E48" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="F48" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="G48" s="49"/>
+      <c r="H48" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="I48" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="I47" s="72">
-        <v>40</v>
-      </c>
-      <c r="J47" s="83">
-        <v>1</v>
-      </c>
-      <c r="K47" s="9"/>
-    </row>
-    <row r="48" spans="1:11" ht="115.5" thickBot="1">
-      <c r="A48" s="6">
-        <v>44</v>
-      </c>
-      <c r="B48" s="90"/>
-      <c r="C48" s="57" t="s">
-        <v>28</v>
-      </c>
-      <c r="D48" s="58" t="s">
-        <v>202</v>
-      </c>
-      <c r="E48" s="59" t="s">
-        <v>29</v>
-      </c>
-      <c r="F48" s="59" t="s">
-        <v>29</v>
-      </c>
-      <c r="G48" s="60"/>
-      <c r="H48" s="61" t="s">
-        <v>31</v>
-      </c>
-      <c r="I48" s="61" t="s">
-        <v>16</v>
-      </c>
-      <c r="J48" s="62">
+      <c r="J48" s="107">
         <v>53</v>
       </c>
       <c r="K48" s="9"/>
     </row>
     <row r="49" spans="1:11" ht="26.25" thickBot="1">
       <c r="A49" s="6">
-        <v>45</v>
-      </c>
-      <c r="B49" s="93" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49" s="81" t="s">
+        <v>118</v>
+      </c>
+      <c r="C49" s="70" t="s">
+        <v>202</v>
+      </c>
+      <c r="D49" s="71" t="s">
+        <v>31</v>
+      </c>
+      <c r="E49" s="71" t="s">
+        <v>31</v>
+      </c>
+      <c r="F49" s="71" t="s">
+        <v>201</v>
+      </c>
+      <c r="G49" s="71" t="s">
+        <v>115</v>
+      </c>
+      <c r="H49" s="71" t="s">
+        <v>115</v>
+      </c>
+      <c r="I49" s="71" t="s">
+        <v>115</v>
+      </c>
+      <c r="J49" s="108">
+        <v>1</v>
+      </c>
+      <c r="K49" s="9"/>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" thickBot="1">
+      <c r="A50" s="111">
+        <v>48</v>
+      </c>
+      <c r="B50" s="82"/>
+      <c r="C50" s="72" t="s">
         <v>119</v>
       </c>
-      <c r="C49" s="102" t="s">
-        <v>205</v>
-      </c>
-      <c r="D49" s="103" t="s">
+      <c r="D50" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="E49" s="103" t="s">
+      <c r="E50" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="F49" s="103" t="s">
-        <v>204</v>
-      </c>
-      <c r="G49" s="103" t="s">
-        <v>116</v>
-      </c>
-      <c r="H49" s="103" t="s">
-        <v>116</v>
-      </c>
-      <c r="I49" s="103" t="s">
-        <v>116</v>
-      </c>
-      <c r="J49" s="104">
-        <v>1</v>
-      </c>
-      <c r="K49" s="9"/>
-    </row>
-    <row r="50" spans="1:11" ht="15.75" thickBot="1">
-      <c r="A50" s="10">
-        <v>46</v>
-      </c>
-      <c r="B50" s="94"/>
-      <c r="C50" s="105" t="s">
-        <v>120</v>
-      </c>
-      <c r="D50" s="106" t="s">
+      <c r="F50" s="73" t="s">
+        <v>119</v>
+      </c>
+      <c r="G50" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="E50" s="106" t="s">
+      <c r="H50" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="F50" s="106" t="s">
-        <v>120</v>
-      </c>
-      <c r="G50" s="106" t="s">
-        <v>31</v>
-      </c>
-      <c r="H50" s="106" t="s">
-        <v>31</v>
-      </c>
-      <c r="I50" s="106" t="s">
+      <c r="I50" s="73" t="s">
         <v>16</v>
       </c>
-      <c r="J50" s="107">
+      <c r="J50" s="109">
         <v>1</v>
       </c>
       <c r="K50" s="9"/>
@@ -3359,7 +3461,7 @@
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="I51" s="7"/>
-      <c r="J51" s="13"/>
+      <c r="J51" s="12"/>
       <c r="K51" s="9"/>
     </row>
     <row r="52" spans="1:11" ht="15.75">
@@ -3367,7 +3469,7 @@
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="I52" s="7"/>
-      <c r="J52" s="13"/>
+      <c r="J52" s="12"/>
       <c r="K52" s="9"/>
     </row>
     <row r="53" spans="1:11">
@@ -3436,15 +3538,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B3:B17"/>
+    <mergeCell ref="B20:B23"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B29:B33"/>
     <mergeCell ref="B34:B42"/>
     <mergeCell ref="B43:B48"/>
     <mergeCell ref="B26:B28"/>
     <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B3:B17"/>
-    <mergeCell ref="B20:B23"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <conditionalFormatting sqref="J3:J8">

</xml_diff>